<commit_message>
fix: correção do getItem
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://suzano-my.sharepoint.com/personal/julianobs_suzano_com_br/Documents/Area Dev/GitHub/UiPath/RoboPedidoDeEmprestimos/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="59" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C7EAA50-5162-4175-9575-729FEB81C34A}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="13_ncr:1_{00D541BD-CB78-4D75-8532-9AD73E8C785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6BAF9F7-5B78-48A2-AE8D-F6A1D7F74DE3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -225,7 +225,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -249,6 +249,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -267,10 +273,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -279,8 +286,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -723,6 +732,7 @@
       <c r="A10" t="s">
         <v>22</v>
       </c>
+      <c r="B10" s="4"/>
       <c r="C10" t="s">
         <v>23</v>
       </c>
@@ -731,6 +741,7 @@
       <c r="A11" t="s">
         <v>24</v>
       </c>
+      <c r="B11" s="4"/>
       <c r="C11" t="s">
         <v>25</v>
       </c>

</xml_diff>